<commit_message>
Correcting start year date part3
</commit_message>
<xml_diff>
--- a/InputData/ccs/CCSTaSC/CCS Transportation and Storage Cost.xlsx
+++ b/InputData/ccs/CCSTaSC/CCS Transportation and Storage Cost.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energyinnovation.sharepoint.com/sites/IndonesiaEPS/Shared Documents/Updated Indonesia InputData files/ccs/CCSTaSC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\ccs\CCSTaSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{6F7C928A-3AAF-49BE-9925-7B059DEE51E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B7ED17A-F837-4C42-9A88-AF373A660732}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60EFB2D1-0228-4AE2-AB1E-78F7476DDC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11205" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -511,111 +511,114 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AF4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="47.1796875" customWidth="1"/>
     <col min="2" max="31" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="B1">
+        <v>2020</v>
+      </c>
+      <c r="C1">
         <v>2021</v>
       </c>
-      <c r="C1">
+      <c r="D1">
         <v>2022</v>
       </c>
-      <c r="D1">
+      <c r="E1">
         <v>2023</v>
       </c>
-      <c r="E1">
+      <c r="F1">
         <v>2024</v>
       </c>
-      <c r="F1">
+      <c r="G1">
         <v>2025</v>
       </c>
-      <c r="G1">
+      <c r="H1">
         <v>2026</v>
       </c>
-      <c r="H1">
+      <c r="I1">
         <v>2027</v>
       </c>
-      <c r="I1">
+      <c r="J1">
         <v>2028</v>
       </c>
-      <c r="J1">
+      <c r="K1">
         <v>2029</v>
       </c>
-      <c r="K1">
+      <c r="L1">
         <v>2030</v>
       </c>
-      <c r="L1">
+      <c r="M1">
         <v>2031</v>
       </c>
-      <c r="M1">
+      <c r="N1">
         <v>2032</v>
       </c>
-      <c r="N1">
+      <c r="O1">
         <v>2033</v>
       </c>
-      <c r="O1">
+      <c r="P1">
         <v>2034</v>
       </c>
-      <c r="P1">
+      <c r="Q1">
         <v>2035</v>
       </c>
-      <c r="Q1">
+      <c r="R1">
         <v>2036</v>
       </c>
-      <c r="R1">
+      <c r="S1">
         <v>2037</v>
       </c>
-      <c r="S1">
+      <c r="T1">
         <v>2038</v>
       </c>
-      <c r="T1">
+      <c r="U1">
         <v>2039</v>
       </c>
-      <c r="U1">
+      <c r="V1">
         <v>2040</v>
       </c>
-      <c r="V1">
+      <c r="W1">
         <v>2041</v>
       </c>
-      <c r="W1">
+      <c r="X1">
         <v>2042</v>
       </c>
-      <c r="X1">
+      <c r="Y1">
         <v>2043</v>
       </c>
-      <c r="Y1">
+      <c r="Z1">
         <v>2044</v>
       </c>
-      <c r="Z1">
+      <c r="AA1">
         <v>2045</v>
       </c>
-      <c r="AA1">
+      <c r="AB1">
         <v>2046</v>
       </c>
-      <c r="AB1">
+      <c r="AC1">
         <v>2047</v>
       </c>
-      <c r="AC1">
+      <c r="AD1">
         <v>2048</v>
       </c>
-      <c r="AD1">
+      <c r="AE1">
         <v>2049</v>
       </c>
-      <c r="AE1">
+      <c r="AF1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
-        <f>About!$B$10*About!$B$11</f>
+        <f>C2</f>
         <v>46.286740359809336</v>
       </c>
       <c r="C2">
@@ -734,8 +737,12 @@
         <f>About!$B$10*About!$B$11</f>
         <v>46.286740359809336</v>
       </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="AF2">
+        <f>About!$B$10*About!$B$11</f>
+        <v>46.286740359809336</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="K4" s="2"/>
     </row>
   </sheetData>
@@ -744,21 +751,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002041A8AB53924247A2770D65450F5227" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="90fff4f083191fe75a03dbd50c7739fc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1659011e-6b88-4225-9a61-aaf33aaf19e8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7fee88694a371868130ae0617c69143c" ns2:_="">
     <xsd:import namespace="1659011e-6b88-4225-9a61-aaf33aaf19e8"/>
@@ -902,24 +894,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5585E82-C794-4536-8A09-03B7BF373BD3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1439C42-A395-413D-8A60-C1AB4FD4A724}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63E5A007-C2FD-45E7-A4B1-27BB10681F10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -935,4 +925,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1439C42-A395-413D-8A60-C1AB4FD4A724}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5585E82-C794-4536-8A09-03B7BF373BD3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>